<commit_message>
20251226: Update Drawing DRC (AR/PR)
</commit_message>
<xml_diff>
--- a/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/Layer_Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D40C962-FF2F-2E4B-8E2D-92DF2C2BCA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56FA8DA6-1D33-DB4F-A457-AC5D5AEF8537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="760" windowWidth="29400" windowHeight="18600" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
+    <workbookView xWindow="860" yWindow="920" windowWidth="30140" windowHeight="18600" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
   <sheets>
     <sheet name="DR (Drawing)" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="239">
   <si>
     <t>Name</t>
   </si>
@@ -678,6 +678,81 @@
   </si>
   <si>
     <t>V1-M2 Emin</t>
+  </si>
+  <si>
+    <t>AC Wmax</t>
+  </si>
+  <si>
+    <t>Table I-2-1</t>
+  </si>
+  <si>
+    <t>PMOS Wmax</t>
+  </si>
+  <si>
+    <t>NMOS Wmax</t>
+  </si>
+  <si>
+    <t>PO Wmax</t>
+  </si>
+  <si>
+    <t>PO(R) Wmax</t>
+  </si>
+  <si>
+    <t>PR.L1</t>
+  </si>
+  <si>
+    <t>PO(R) Lmin</t>
+  </si>
+  <si>
+    <t>PO(R) Lmax</t>
+  </si>
+  <si>
+    <t>AR.W2</t>
+  </si>
+  <si>
+    <t>AR Wmax</t>
+  </si>
+  <si>
+    <t>AR.L1</t>
+  </si>
+  <si>
+    <t>AR.L2</t>
+  </si>
+  <si>
+    <t>AR Lmin</t>
+  </si>
+  <si>
+    <t>AR Lmax</t>
+  </si>
+  <si>
+    <t>AR.XT</t>
+  </si>
+  <si>
+    <t>AR corner cut</t>
+  </si>
+  <si>
+    <t>CR.W1</t>
+  </si>
+  <si>
+    <t>CR.W2</t>
+  </si>
+  <si>
+    <t>CR.AT</t>
+  </si>
+  <si>
+    <t>CR.AS</t>
+  </si>
+  <si>
+    <t>CO(RR) Wmin</t>
+  </si>
+  <si>
+    <t>CO(RR) Width</t>
+  </si>
+  <si>
+    <t>CO(RR)-AR(Top) Emin</t>
+  </si>
+  <si>
+    <t>CO(RR)-AR(Side) Emin</t>
   </si>
 </sst>
 </file>
@@ -1545,7 +1620,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4478C0F2-BA21-8B4B-B7C2-220C0E7FA6A8}">
-  <dimension ref="B2:E85"/>
+  <dimension ref="B2:E105"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.6640625" style="1" customWidth="1"/>
@@ -1712,207 +1787,209 @@
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B13" s="13" t="s">
-        <v>27</v>
+        <v>223</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>35</v>
+        <v>224</v>
       </c>
       <c r="D13" s="15">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>40</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B14" s="13" t="s">
-        <v>28</v>
+        <v>225</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>36</v>
+        <v>227</v>
       </c>
       <c r="D14" s="15">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>39</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B15" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>228</v>
+      </c>
+      <c r="D15" s="15">
+        <v>100</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B16" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="15">
+        <v>4</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B17" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D17" s="15">
+        <v>10</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B18" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="14" t="s">
+      <c r="C18" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="15">
+      <c r="D18" s="15">
         <v>5</v>
       </c>
-      <c r="E15" s="13" t="s">
+      <c r="E18" s="13" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B16" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="10">
-        <v>4</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B17" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E17" s="8"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B18" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>57</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E18" s="8"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B19" s="8" t="s">
-        <v>46</v>
+        <v>30</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="D19" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E19" s="8"/>
+        <v>37</v>
+      </c>
+      <c r="D19" s="10">
+        <v>4</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B20" s="8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D20" s="10">
-        <v>3</v>
+        <v>28.5</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>60</v>
+        <v>215</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B21" s="8" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>49</v>
+        <v>214</v>
       </c>
       <c r="D21" s="10">
-        <v>2.8</v>
+        <v>120</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>61</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B22" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B23" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B24" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D24" s="10">
+        <v>3</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B25" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D25" s="10">
+        <v>2.8</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B26" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C26" s="9" t="s">
         <v>169</v>
       </c>
-      <c r="D22" s="10"/>
-      <c r="E22" s="8"/>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B23" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="D23" s="15">
-        <v>1.4</v>
-      </c>
-      <c r="E23" s="13" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B24" s="13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C24" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="15">
-        <v>1.4</v>
-      </c>
-      <c r="E24" s="13" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B25" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C25" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="D25" s="15">
-        <v>2.8</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B26" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="C26" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="D26" s="15">
-        <v>3.4</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B27" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="D27" s="15">
-        <v>7</v>
-      </c>
-      <c r="E27" s="13" t="s">
-        <v>31</v>
+      <c r="D26" s="10"/>
+      <c r="E26" s="8"/>
+    </row>
+    <row r="27" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B28" s="13" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="C28" s="14" t="s">
         <v>66</v>
@@ -1926,723 +2003,993 @@
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B29" s="13" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>58</v>
+        <v>67</v>
+      </c>
+      <c r="D29" s="15">
+        <v>1.4</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B30" s="13" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D30" s="15">
         <v>2.8</v>
       </c>
       <c r="E30" s="13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B31" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" s="15">
+        <v>3.4</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B32" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="D32" s="15">
+        <v>60</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B33" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="D33" s="15">
+        <v>7</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B34" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C34" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" s="15">
+        <v>1.4</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B35" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B36" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C36" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="D36" s="15">
+        <v>2.8</v>
+      </c>
+      <c r="E36" s="13" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="31" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B31" s="13" t="s">
+    <row r="37" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="C31" s="14" t="s">
+      <c r="C37" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D37" s="15">
         <v>2.8</v>
       </c>
-      <c r="E31" s="13" t="s">
+      <c r="E37" s="13" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B32" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="C32" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="D32" s="10">
-        <v>1.4</v>
-      </c>
-      <c r="E32" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B33" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C33" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="D33" s="10">
-        <v>1.4</v>
-      </c>
-      <c r="E33" s="8" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B34" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="D34" s="10">
-        <v>2.8</v>
-      </c>
-      <c r="E34" s="8" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B35" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="D35" s="10">
-        <v>3.4</v>
-      </c>
-      <c r="E35" s="8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B36" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C36" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="D36" s="10">
-        <v>5</v>
-      </c>
-      <c r="E36" s="8" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B37" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="C37" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="D37" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="E37" s="8" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B38" s="8" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="C38" s="9" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="D38" s="10">
+        <v>1.4</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B39" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39" s="10">
+        <v>1.4</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B40" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D40" s="10">
         <v>2.8</v>
       </c>
-      <c r="E38" s="8" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="39" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="D39" s="10">
-        <v>2.8</v>
-      </c>
-      <c r="E39" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B40" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="D40" s="15">
-        <v>1</v>
-      </c>
-      <c r="E40" s="13" t="s">
-        <v>171</v>
+      <c r="E40" s="8" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B41" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C41" s="14" t="s">
-        <v>106</v>
-      </c>
-      <c r="D41" s="15">
-        <v>1.2</v>
-      </c>
-      <c r="E41" s="13" t="s">
-        <v>172</v>
+      <c r="B41" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="D41" s="10">
+        <v>3.4</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B42" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C42" s="14" t="s">
-        <v>107</v>
-      </c>
-      <c r="D42" s="15">
-        <v>0.4</v>
-      </c>
-      <c r="E42" s="13" t="s">
-        <v>173</v>
+      <c r="B42" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="C42" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="D42" s="10">
+        <v>60</v>
+      </c>
+      <c r="E42" s="8" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B43" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="C43" s="14" t="s">
-        <v>108</v>
-      </c>
-      <c r="D43" s="15">
-        <v>0.4</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>174</v>
+      <c r="B43" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D43" s="10">
+        <v>5</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B44" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="C44" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="D44" s="15">
-        <v>1.2</v>
-      </c>
-      <c r="E44" s="13" t="s">
-        <v>175</v>
+      <c r="B44" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="E44" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B45" s="8" t="s">
-        <v>109</v>
+        <v>85</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>113</v>
+        <v>82</v>
       </c>
       <c r="D45" s="10">
+        <v>2.8</v>
+      </c>
+      <c r="E45" s="8" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="46" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B46" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="C46" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D46" s="10">
+        <v>2.8</v>
+      </c>
+      <c r="E46" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="47" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B47" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C47" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D47" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B48" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="D48" s="15">
         <v>1</v>
       </c>
-      <c r="E45" s="8" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="46" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B46" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="D46" s="10">
-        <v>1</v>
-      </c>
-      <c r="E46" s="8" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B47" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>112</v>
-      </c>
-      <c r="D47" s="10">
+      <c r="E48" s="13" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B49" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C49" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="D49" s="15">
+        <v>30</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B50" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C50" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D50" s="15">
         <v>1.2</v>
       </c>
-      <c r="E47" s="8" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B48" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="D48" s="10">
-        <v>0.8</v>
-      </c>
-      <c r="E48" s="8" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="49" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B49" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="C49" s="9" t="s">
-        <v>118</v>
-      </c>
-      <c r="D49" s="10">
-        <v>0.8</v>
-      </c>
-      <c r="E49" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B50" s="8" t="s">
-        <v>119</v>
-      </c>
-      <c r="C50" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="D50" s="10">
-        <v>1</v>
-      </c>
-      <c r="E50" s="8" t="s">
-        <v>181</v>
+      <c r="E50" s="13" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B51" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="D51" s="10">
-        <v>0.8</v>
-      </c>
-      <c r="E51" s="8" t="s">
-        <v>182</v>
+      <c r="B51" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C51" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="D51" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B52" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="C52" s="9" t="s">
-        <v>124</v>
-      </c>
-      <c r="D52" s="10">
-        <v>1.2</v>
-      </c>
-      <c r="E52" s="8" t="s">
-        <v>183</v>
+      <c r="B52" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C52" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="D52" s="15">
+        <v>0.4</v>
+      </c>
+      <c r="E52" s="13" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B53" s="13" t="s">
-        <v>160</v>
+        <v>104</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D53" s="15">
+        <v>1.2</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B54" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="D54" s="10">
         <v>1</v>
       </c>
-      <c r="E53" s="13" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="54" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B54" s="13" t="s">
-        <v>161</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="D54" s="15">
-        <v>2</v>
-      </c>
-      <c r="E54" s="13" t="s">
-        <v>185</v>
+      <c r="E54" s="8" t="s">
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B55" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="C55" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="D55" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="E55" s="13"/>
+      <c r="B55" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="D55" s="10">
+        <v>1</v>
+      </c>
+      <c r="E55" s="8" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B56" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="C56" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="D56" s="15"/>
-      <c r="E56" s="13"/>
+      <c r="B56" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D56" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="E56" s="8" t="s">
+        <v>178</v>
+      </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B57" s="13" t="s">
-        <v>168</v>
-      </c>
-      <c r="C57" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="D57" s="15"/>
-      <c r="E57" s="13"/>
+      <c r="B57" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="D57" s="10">
+        <v>0.8</v>
+      </c>
+      <c r="E57" s="8" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B58" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="C58" s="14" t="s">
-        <v>204</v>
-      </c>
-      <c r="D58" s="15">
+      <c r="B58" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="C58" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="D58" s="10">
+        <v>0.8</v>
+      </c>
+      <c r="E58" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B59" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="D59" s="10">
         <v>1</v>
       </c>
-      <c r="E58" s="13" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="59" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B59" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="C59" s="14" t="s">
-        <v>205</v>
-      </c>
-      <c r="D59" s="15">
-        <v>2</v>
-      </c>
-      <c r="E59" s="13" t="s">
-        <v>207</v>
+      <c r="E59" s="8" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B60" s="8" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C60" s="9" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D60" s="10">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B61" s="8" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D61" s="10">
         <v>1.2</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="62" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B62" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="C62" s="9" t="s">
-        <v>131</v>
-      </c>
-      <c r="D62" s="10">
-        <v>2.9</v>
-      </c>
-      <c r="E62" s="8" t="s">
-        <v>188</v>
+        <v>183</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B62" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C62" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D62" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B63" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="C63" s="9" t="s">
-        <v>132</v>
-      </c>
-      <c r="D63" s="10">
-        <v>1.2</v>
-      </c>
-      <c r="E63" s="8" t="s">
-        <v>189</v>
+      <c r="B63" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="C63" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="D63" s="15">
+        <v>1</v>
+      </c>
+      <c r="E63" s="13" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B64" s="8" t="s">
-        <v>208</v>
-      </c>
-      <c r="C64" s="9" t="s">
-        <v>210</v>
-      </c>
-      <c r="D64" s="10">
-        <v>1</v>
-      </c>
-      <c r="E64" s="8" t="s">
-        <v>197</v>
+      <c r="B64" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="C64" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D64" s="15">
+        <v>2</v>
+      </c>
+      <c r="E64" s="13" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B65" s="8" t="s">
-        <v>209</v>
-      </c>
-      <c r="C65" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="D65" s="10">
-        <v>1.2</v>
-      </c>
-      <c r="E65" s="8" t="s">
-        <v>189</v>
-      </c>
+      <c r="B65" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="C65" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="D65" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="E65" s="13"/>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B66" s="13" t="s">
-        <v>133</v>
+        <v>167</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>136</v>
-      </c>
-      <c r="D66" s="15">
-        <v>1.8</v>
-      </c>
-      <c r="E66" s="13" t="s">
-        <v>190</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="D66" s="15"/>
+      <c r="E66" s="13"/>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B67" s="13" t="s">
-        <v>134</v>
+        <v>168</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>137</v>
-      </c>
-      <c r="D67" s="15">
-        <v>1.4</v>
-      </c>
-      <c r="E67" s="13" t="s">
-        <v>191</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="D67" s="15"/>
+      <c r="E67" s="13"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B68" s="13" t="s">
-        <v>133</v>
+        <v>202</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>138</v>
+        <v>204</v>
       </c>
       <c r="D68" s="15">
-        <v>10</v>
+        <v>2.8</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B69" s="13" t="s">
-        <v>135</v>
+        <v>202</v>
       </c>
       <c r="C69" s="14" t="s">
-        <v>139</v>
+        <v>204</v>
       </c>
       <c r="D69" s="15">
+        <v>4</v>
+      </c>
+      <c r="E69" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="70" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B70" s="13" t="s">
+        <v>202</v>
+      </c>
+      <c r="C70" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="D70" s="15">
+        <v>20</v>
+      </c>
+      <c r="E70" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="71" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B71" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="C71" s="14" t="s">
+        <v>221</v>
+      </c>
+      <c r="D71" s="15">
+        <v>20</v>
+      </c>
+      <c r="E71" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="72" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B72" s="13" t="s">
+        <v>220</v>
+      </c>
+      <c r="C72" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="D72" s="15">
+        <v>100</v>
+      </c>
+      <c r="E72" s="13" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="73" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B73" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="C73" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="D73" s="15">
         <v>2</v>
       </c>
-      <c r="E69" s="13" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="70" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B70" s="8" t="s">
-        <v>140</v>
-      </c>
-      <c r="C70" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="D70" s="10">
-        <v>1.4</v>
-      </c>
-      <c r="E70" s="8" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="71" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B71" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="C71" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="D71" s="10">
-        <v>1.5</v>
-      </c>
-      <c r="E71" s="8" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="72" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B72" s="8" t="s">
-        <v>142</v>
-      </c>
-      <c r="C72" s="9" t="s">
-        <v>150</v>
-      </c>
-      <c r="D72" s="10">
-        <v>1</v>
-      </c>
-      <c r="E72" s="8" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="73" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B73" s="8" t="s">
-        <v>212</v>
-      </c>
-      <c r="C73" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="D73" s="10">
-        <v>1</v>
-      </c>
-      <c r="E73" s="8" t="s">
-        <v>196</v>
+      <c r="E73" s="13" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B74" s="8" t="s">
-        <v>143</v>
+        <v>229</v>
       </c>
       <c r="C74" s="9" t="s">
-        <v>151</v>
+        <v>230</v>
       </c>
       <c r="D74" s="10">
-        <v>1.2</v>
-      </c>
-      <c r="E74" s="8" t="s">
-        <v>199</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E74" s="8"/>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B75" s="8" t="s">
-        <v>144</v>
-      </c>
-      <c r="C75" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="D75" s="10">
+      <c r="B75" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="C75" s="14" t="s">
+        <v>236</v>
+      </c>
+      <c r="D75" s="15">
         <v>1</v>
       </c>
-      <c r="E75" s="8" t="s">
-        <v>200</v>
-      </c>
+      <c r="E75" s="13"/>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B76" s="8" t="s">
-        <v>145</v>
-      </c>
-      <c r="C76" s="9" t="s">
-        <v>153</v>
-      </c>
-      <c r="D76" s="10">
-        <v>1.4</v>
-      </c>
-      <c r="E76" s="8" t="s">
-        <v>201</v>
-      </c>
+      <c r="B76" s="13" t="s">
+        <v>232</v>
+      </c>
+      <c r="C76" s="14" t="s">
+        <v>235</v>
+      </c>
+      <c r="D76" s="15">
+        <v>1</v>
+      </c>
+      <c r="E76" s="13"/>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B77" s="13" t="s">
-        <v>146</v>
+        <v>233</v>
       </c>
       <c r="C77" s="14" t="s">
-        <v>154</v>
+        <v>237</v>
       </c>
       <c r="D77" s="15">
-        <v>3</v>
-      </c>
-      <c r="E77" s="13" t="s">
-        <v>194</v>
-      </c>
+        <v>1.5</v>
+      </c>
+      <c r="E77" s="13"/>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.2">
       <c r="B78" s="13" t="s">
+        <v>234</v>
+      </c>
+      <c r="C78" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="D78" s="15">
+        <v>1</v>
+      </c>
+      <c r="E78" s="13"/>
+    </row>
+    <row r="79" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B79" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="C79" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D79" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="80" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B80" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="C80" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="D80" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="E80" s="8" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="81" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B81" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="C81" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D81" s="10">
+        <v>2.9</v>
+      </c>
+      <c r="E81" s="8" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="82" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B82" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="C82" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="D82" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="E82" s="8" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="83" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B83" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="C83" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="D83" s="10">
+        <v>1</v>
+      </c>
+      <c r="E83" s="8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="84" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B84" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="C84" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="D84" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="E84" s="8" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="85" spans="2:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B85" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="C85" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D85" s="16" t="s">
+        <v>156</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="86" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B86" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="C86" s="14" t="s">
+        <v>136</v>
+      </c>
+      <c r="D86" s="15">
+        <v>1.8</v>
+      </c>
+      <c r="E86" s="13" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="87" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B87" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="C87" s="14" t="s">
+        <v>137</v>
+      </c>
+      <c r="D87" s="15">
+        <v>1.4</v>
+      </c>
+      <c r="E87" s="13" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="88" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B88" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="C88" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="D88" s="15">
+        <v>10</v>
+      </c>
+      <c r="E88" s="13" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B89" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="C89" s="14" t="s">
+        <v>139</v>
+      </c>
+      <c r="D89" s="15">
+        <v>2</v>
+      </c>
+      <c r="E89" s="13" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="90" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B90" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C90" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="D90" s="10">
+        <v>1.4</v>
+      </c>
+      <c r="E90" s="8" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="91" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B91" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="C91" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="D91" s="10">
+        <v>1.5</v>
+      </c>
+      <c r="E91" s="8" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="92" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B92" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="C92" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D92" s="10">
+        <v>1</v>
+      </c>
+      <c r="E92" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="93" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B93" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="C93" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="D93" s="10">
+        <v>1</v>
+      </c>
+      <c r="E93" s="8" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="94" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B94" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="C94" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="D94" s="10">
+        <v>1.2</v>
+      </c>
+      <c r="E94" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="95" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B95" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="C95" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="D95" s="10">
+        <v>1</v>
+      </c>
+      <c r="E95" s="8" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="96" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B96" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C96" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D96" s="10">
+        <v>1.4</v>
+      </c>
+      <c r="E96" s="8" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="97" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B97" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="C97" s="14" t="s">
+        <v>154</v>
+      </c>
+      <c r="D97" s="15">
+        <v>3</v>
+      </c>
+      <c r="E97" s="13" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="98" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B98" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="C78" s="14" t="s">
+      <c r="C98" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="D78" s="15">
+      <c r="D98" s="15">
         <v>2</v>
       </c>
-      <c r="E78" s="13" t="s">
+      <c r="E98" s="13" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="80" spans="2:5" x14ac:dyDescent="0.2">
-      <c r="B80" s="4"/>
-      <c r="C80" s="6"/>
-      <c r="D80" s="5"/>
-    </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B81" s="4"/>
-      <c r="C81" s="6"/>
-      <c r="D81" s="5"/>
-    </row>
-    <row r="82" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B82" s="4"/>
-      <c r="C82" s="6"/>
-      <c r="D82" s="5"/>
-    </row>
-    <row r="83" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B83" s="4"/>
-      <c r="C83" s="6"/>
-      <c r="D83" s="5"/>
-    </row>
-    <row r="84" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B84" s="4"/>
-      <c r="C84" s="6"/>
-      <c r="D84" s="5"/>
-    </row>
-    <row r="85" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B85" s="4"/>
-      <c r="C85" s="6"/>
-      <c r="D85" s="5"/>
+    <row r="100" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B100" s="4"/>
+      <c r="C100" s="6"/>
+      <c r="D100" s="5"/>
+    </row>
+    <row r="101" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B101" s="4"/>
+      <c r="C101" s="6"/>
+      <c r="D101" s="5"/>
+    </row>
+    <row r="102" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B102" s="4"/>
+      <c r="C102" s="6"/>
+      <c r="D102" s="5"/>
+    </row>
+    <row r="103" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B103" s="4"/>
+      <c r="C103" s="6"/>
+      <c r="D103" s="5"/>
+    </row>
+    <row r="104" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B104" s="4"/>
+      <c r="C104" s="6"/>
+      <c r="D104" s="5"/>
+    </row>
+    <row r="105" spans="2:5" x14ac:dyDescent="0.2">
+      <c r="B105" s="4"/>
+      <c r="C105" s="6"/>
+      <c r="D105" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
20251230: Use "PMOS/NMOS" for Endcap.
</commit_message>
<xml_diff>
--- a/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
+++ b/Document/Layer_Tables/TR-1um_Drawing_Layer_DR_Table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/okamura/Library/CloudStorage/Dropbox/91_OpenPDK/TR-1um/Document/Layer_Tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F6DBB7F-9449-CC49-A39F-AF81CB24943E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23B36F77-5DF6-D24A-9A7E-746FCC254D02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12080" yWindow="2880" windowWidth="29420" windowHeight="18600" xr2:uid="{7F1200E8-B51D-9446-A5CE-CEA05B5231B7}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="225">
   <si>
     <t>WN.W1</t>
   </si>
@@ -660,12 +660,6 @@
   </si>
   <si>
     <t>AN-PO</t>
-  </si>
-  <si>
-    <t>PO&amp;AP</t>
-  </si>
-  <si>
-    <t>PO&amp;AN</t>
   </si>
   <si>
     <t>ECmin</t>
@@ -1819,7 +1813,7 @@
         <v>158</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>185</v>
@@ -2307,7 +2301,7 @@
         <v>149</v>
       </c>
       <c r="D30" s="11" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="E30" s="5" t="s">
         <v>179</v>
@@ -2446,7 +2440,7 @@
         <v>152</v>
       </c>
       <c r="D37" s="13" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E37" s="8" t="s">
         <v>150</v>
@@ -2656,7 +2650,7 @@
         <v>155</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="E47" s="5" t="s">
         <v>150</v>
@@ -2679,7 +2673,7 @@
         <v>154</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E48" s="5" t="s">
         <v>147</v>
@@ -2896,44 +2890,44 @@
     </row>
     <row r="59" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B59" s="8" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C59" s="13" t="s">
-        <v>208</v>
+        <v>152</v>
       </c>
       <c r="D59" s="13" t="s">
         <v>157</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F59" s="9">
         <v>1.2</v>
       </c>
       <c r="G59" s="9"/>
       <c r="H59" s="8" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="60" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B60" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C60" s="13" t="s">
-        <v>209</v>
+        <v>155</v>
       </c>
       <c r="D60" s="13" t="s">
         <v>157</v>
       </c>
       <c r="E60" s="8" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F60" s="9">
         <v>1.2</v>
       </c>
       <c r="G60" s="9"/>
       <c r="H60" s="8" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="61" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -3141,10 +3135,10 @@
         <v>20</v>
       </c>
       <c r="C71" s="13" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D71" s="13" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E71" s="8" t="s">
         <v>146</v>
@@ -3164,10 +3158,10 @@
         <v>125</v>
       </c>
       <c r="C72" s="13" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D72" s="13" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E72" s="8" t="s">
         <v>150</v>
@@ -3301,10 +3295,10 @@
         <v>121</v>
       </c>
       <c r="C79" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D79" s="11" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="E79" s="5" t="s">
         <v>146</v>
@@ -3321,13 +3315,13 @@
     </row>
     <row r="80" spans="2:8" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B80" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C80" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D80" s="11" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E80" s="5" t="s">
         <v>150</v>
@@ -3347,10 +3341,10 @@
         <v>122</v>
       </c>
       <c r="C81" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D81" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E81" s="5" t="s">
         <v>145</v>
@@ -3626,7 +3620,7 @@
         <v>165</v>
       </c>
       <c r="D95" s="11" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="E95" s="5" t="s">
         <v>160</v>

</xml_diff>